<commit_message>
Fix ConceptMap validation errors reported by QA fd105af2800ec5fe475c78e40e5e156cc2ad756b
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
+++ b/fix-target-codes-and-display/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
@@ -9,12 +9,14 @@
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
     <sheet name="Mapping Table 0" r:id="rId4" sheetId="2"/>
     <sheet name="Mapping Table 1" r:id="rId5" sheetId="3"/>
+    <sheet name="Mapping Table 2" r:id="rId6" sheetId="4"/>
+    <sheet name="Mapping Table 3" r:id="rId7" sheetId="5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -37,6 +39,9 @@
     <t>Name</t>
   </si>
   <si>
+    <t>FRAdvanceDirectiveLMCDAFHIR</t>
+  </si>
+  <si>
     <t>Title</t>
   </si>
   <si>
@@ -52,10 +57,13 @@
     <t>Experimental</t>
   </si>
   <si>
+    <t>false</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T15:24:46+00:00</t>
+    <t>2026-08-21T08:13:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -157,70 +165,70 @@
     <t>Observation.text</t>
   </si>
   <si>
-    <t>FRLMAdvanceDirective.attachment.url</t>
+    <t>FRLMAdvanceDirective.attachment</t>
+  </si>
+  <si>
+    <t>Observation.entryRelationship.observationMedia</t>
+  </si>
+  <si>
+    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-advance-directive-document|0.1.0</t>
+  </si>
+  <si>
+    <t>Consent</t>
+  </si>
+  <si>
+    <t>FRAdvanceDirectiveDocument</t>
+  </si>
+  <si>
+    <t>Consent.identifier</t>
+  </si>
+  <si>
+    <t>Consent.provision.code</t>
+  </si>
+  <si>
+    <t>Consent.status</t>
+  </si>
+  <si>
+    <t>FRLMAdvanceDirective.date</t>
+  </si>
+  <si>
+    <t>Consent.dateTime</t>
+  </si>
+  <si>
+    <t>Consent.provision.type</t>
+  </si>
+  <si>
+    <t>Consent.source[x]</t>
+  </si>
+  <si>
+    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMAttachment|0.1.0</t>
+  </si>
+  <si>
+    <t>FRLMAttachment.url</t>
   </si>
   <si>
     <t>Observation.reference.externalDocument.text.reference</t>
   </si>
   <si>
-    <t>FRLMAdvanceDirective.attachment</t>
-  </si>
-  <si>
-    <t>Observation.entryRelationship.observationMedia</t>
-  </si>
-  <si>
-    <t>FRLMAdvanceDirective.attachment.header.identifier</t>
+    <t>FRLMAttachment.header.identifier</t>
   </si>
   <si>
     <t>Observation.entryRelationship.observationMedia.id</t>
   </si>
   <si>
-    <t>FRLMAdvanceDirective.attachment.data</t>
+    <t>FRLMAttachment.data</t>
   </si>
   <si>
     <t>Observation.entryRelationship.observationMedia.value</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-advance-directive-document|0.1.0</t>
-  </si>
-  <si>
-    <t>Consent</t>
-  </si>
-  <si>
-    <t>FRAdvanceDirectiveDocument</t>
-  </si>
-  <si>
-    <t>Consent.identifier</t>
-  </si>
-  <si>
-    <t>Consent.provision.code</t>
-  </si>
-  <si>
-    <t>Consent.provision.code.text</t>
-  </si>
-  <si>
-    <t>Consent.status</t>
-  </si>
-  <si>
-    <t>FRLMAdvanceDirective.date</t>
-  </si>
-  <si>
-    <t>Consent.dateTime</t>
-  </si>
-  <si>
-    <t>Consent.provision.type</t>
-  </si>
-  <si>
-    <t>Consent.sourceReference</t>
-  </si>
-  <si>
-    <t>Consent.sourceAttachment</t>
-  </si>
-  <si>
-    <t>Consent.sourceAttachment.id</t>
-  </si>
-  <si>
-    <t>Consent.sourceAttachment.data</t>
+    <t>Consent.source[x].url</t>
+  </si>
+  <si>
+    <t>Consent.source[x].id</t>
+  </si>
+  <si>
+    <t>Consent.source[x].data</t>
   </si>
 </sst>
 </file>
@@ -389,79 +397,83 @@
       <c r="A4" t="s" s="2">
         <v>6</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" t="s" s="2">
+        <v>7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>11</v>
-      </c>
-      <c r="B7" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2"/>
     </row>
@@ -472,187 +484,148 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
         <v>27</v>
-      </c>
-      <c r="E1" t="s" s="1">
-        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E10" s="2"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s" s="2">
-        <v>50</v>
-      </c>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="2">
-        <v>51</v>
-      </c>
-      <c r="B12" s="2"/>
-      <c r="C12" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s" s="2">
-        <v>52</v>
-      </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s" s="2">
-        <v>54</v>
-      </c>
-      <c r="E13" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -661,187 +634,301 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
         <v>27</v>
-      </c>
-      <c r="E1" t="s" s="1">
-        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s" s="2">
+        <v>60</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
         <v>32</v>
       </c>
-      <c r="D9" t="s" s="2">
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>62</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>63</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
         <v>64</v>
       </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="2">
-        <v>47</v>
-      </c>
-      <c r="B10" s="2"/>
-      <c r="C10" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D10" t="s" s="2">
+      <c r="B4" s="2"/>
+      <c r="C4" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="2">
         <v>65</v>
       </c>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="2">
-        <v>49</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D11" t="s" s="2">
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
         <v>66</v>
       </c>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="2">
+      <c r="B5" s="2"/>
+      <c r="C5" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>67</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s" s="2">
         <v>51</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s" s="2">
-        <v>67</v>
-      </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="2">
-        <v>53</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="D13" t="s" s="2">
+      <c r="E2" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>62</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s" s="2">
         <v>68</v>
       </c>
-      <c r="E13" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>69</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>66</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="E5" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Fix ConceptMap validation errors reported by QA f2a52b7f3d313b4179eee58ee6a58b9f2479e383
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
+++ b/fix-target-codes-and-display/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T08:13:05+00:00</t>
+    <t>2026-08-23T21:45:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -222,13 +222,13 @@
     <t>Observation.entryRelationship.observationMedia.value</t>
   </si>
   <si>
-    <t>Consent.source[x].url</t>
-  </si>
-  <si>
-    <t>Consent.source[x].id</t>
-  </si>
-  <si>
-    <t>Consent.source[x].data</t>
+    <t>Consent.source[x]:sourceAttachment.url</t>
+  </si>
+  <si>
+    <t>Consent.source[x]:sourceAttachment.id</t>
+  </si>
+  <si>
+    <t>Consent.source[x]:sourceAttachment.data</t>
   </si>
 </sst>
 </file>

</xml_diff>